<commit_message>
Add savings-lever sheet and card-price comparison
New "Sparhebel" sheet lists 15 additional ways to lower the price,
grouped into purchase-price alternatives, stackable discounts, and
avoided costs. Each lever has an editable estimate and a Ja/Nein/Prüfen
switch feeding a secured total and a best-case total; mutually
exclusive levers default to "Nein" so the best case stays realistic.

Also adds a card-price comparison table on "PSN-Karten" (45.49 down to
37.50 per 50 EUR) and two new rows on "Szenarien".

Researched and incorporated: 899.99 EUR is the confirmed list price
after the April 2026 increase, the detachable CFI-ZDD1 disc drive is
shared between PS5 Slim and PS5 Pro, retail prices run well below list,
and PSN credit is widely available below the 45.49 EUR assumed so far.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012kmdvoPfwJH2aPUXAdWVWm
</commit_message>
<xml_diff>
--- a/PS5_Pro_Kaufkalkulation.xlsx
+++ b/PS5_Pro_Kaufkalkulation.xlsx
@@ -10,7 +10,8 @@
   <sheets>
     <sheet name="Kalkulation" sheetId="1" state="visible" r:id="rId3"/>
     <sheet name="PSN-Karten" sheetId="2" state="visible" r:id="rId4"/>
-    <sheet name="Szenarien" sheetId="3" state="visible" r:id="rId5"/>
+    <sheet name="Sparhebel" sheetId="3" state="visible" r:id="rId5"/>
+    <sheet name="Szenarien" sheetId="4" state="visible" r:id="rId6"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -22,12 +23,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="117" uniqueCount="112">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="226" uniqueCount="206">
   <si>
     <t xml:space="preserve">PlayStation 5 Pro — Kaufkalkulation</t>
   </si>
   <si>
-    <t xml:space="preserve">Alle Beträge in Euro · Blaue Zahlen = Eingaben, die du ändern kannst · Schwarze Zahlen = berechnet</t>
+    <t xml:space="preserve">Alle Beträge in Euro · Blaue Zahlen = Eingaben, die du ändern kannst · Schwarze Zahlen = berechnet · Grüne Zahlen = von einem anderen Blatt</t>
   </si>
   <si>
     <t xml:space="preserve">1. Eingaben</t>
@@ -45,7 +46,7 @@
     <t xml:space="preserve">Listenpreis PS5 Pro</t>
   </si>
   <si>
-    <t xml:space="preserve">Du hast "899 €" genannt — deine Zwischenwerte (482,99 / 432,99) gehen nur mit 899,99 € auf. Bei glatt 899,00 € hier überschreiben.</t>
+    <t xml:space="preserve">Bestätigt: 899,99 € ist die offizielle UVP seit der Preiserhöhung vom 02.04.2026. Deine Zwischenwerte 482,99 / 432,99 gehen damit exakt auf.</t>
   </si>
   <si>
     <t xml:space="preserve">Warenkorb-Rabatt (sofort)</t>
@@ -63,7 +64,7 @@
     <t xml:space="preserve">Eintausch-Bonus von PlayStation</t>
   </si>
   <si>
-    <t xml:space="preserve">Zusätzlicher Gutschein, nur bei Eintausch (nicht bei Privatverkauf).</t>
+    <t xml:space="preserve">Zusätzlicher Gutschein, nur bei Eintausch — nicht bei Privatverkauf.</t>
   </si>
   <si>
     <t xml:space="preserve">PSN-Karte — Nennwert</t>
@@ -72,10 +73,10 @@
     <t xml:space="preserve">Guthaben, das die Karte auf dem Konto gutschreibt.</t>
   </si>
   <si>
-    <t xml:space="preserve">PSN-Karte — Kaufpreis</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Was du für die Karte bezahlst.</t>
+    <t xml:space="preserve">PSN-Karte — dein Kaufpreis</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dein gefundener Preis. Es geht deutlich günstiger — siehe Blatt "PSN-Karten".</t>
   </si>
   <si>
     <t xml:space="preserve">2. Rechenweg bis zum Eigenanteil</t>
@@ -111,7 +112,7 @@
     <t xml:space="preserve">3. Zahlung mit vergünstigten PSN-Guthabenkarten</t>
   </si>
   <si>
-    <t xml:space="preserve">Jede Karte bringt 50 € Guthaben und kostet nur 45,49 € — Details und Stückzahlen auf dem Blatt "PSN-Karten".</t>
+    <t xml:space="preserve">Details und Stückzahlen auf dem Blatt "PSN-Karten".</t>
   </si>
   <si>
     <t xml:space="preserve">Ersparnis pro Karte</t>
@@ -123,6 +124,9 @@
     <t xml:space="preserve">Rabatt in Prozent</t>
   </si>
   <si>
+    <t xml:space="preserve">Zum Vergleich: seriöse Anbieter liegen bei 12-18 %.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Variante A — nur volle Karten, Rest bar</t>
   </si>
   <si>
@@ -159,7 +163,7 @@
     <t xml:space="preserve">Barwert des Bonus, falls PSN-Guthaben</t>
   </si>
   <si>
-    <t xml:space="preserve">Ein 50-€-PSN-Gutschein ist real nur 45,49 € wert — so viel kostet er als Karte.</t>
+    <t xml:space="preserve">Ein 50-€-PSN-Gutschein ist real nur so viel wert, wie er als Karte kostet.</t>
   </si>
   <si>
     <t xml:space="preserve">Eintausch bar bewertet</t>
@@ -171,19 +175,22 @@
     <t xml:space="preserve">5. Wichtige Hinweise</t>
   </si>
   <si>
+    <t xml:space="preserve">•  KRITISCH ZUERST PRÜFEN: Kann die Konsole überhaupt mit PSN-Guthaben bezahlt werden? Bei PlayStation Direct gilt Wallet-Guthaben üblicherweise nur für Spiele, Add-ons und Abos, nicht für Hardware. Klappt es nicht, fällt die gesamte Kartenrechnung weg und du bleibst beim Eigenanteil aus Zeile 20.</t>
+  </si>
+  <si>
     <t xml:space="preserve">•  Die 372 € und der 50-€-Bonus gehören zum selben Vorgang: Du kannst die Slim entweder eintauschen ODER privat verkaufen, nicht beides.</t>
   </si>
   <si>
-    <t xml:space="preserve">•  Prüfe vor dem Kauf, ob der Händler Hardware überhaupt mit PSN-Guthaben bezahlen lässt — bei PlayStation Direct gilt Wallet-Guthaben üblicherweise nur für Spiele und Abos, nicht für Konsolen.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">•  Ist der 50-€-Bonus ein PSN-Gutschein statt Bargeld, sinkt sein echter Wert auf 45,49 € (Zeile 34).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">•  Alle Preise stammen aus deinen Angaben vom 12.08.2026 und sind keine geprüften Händlerpreise.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PSN-Guthabenkarten — wie viele lohnen sich?</t>
+    <t xml:space="preserve">•  Ist der 50-€-Bonus ein PSN-Gutschein statt Bargeld, sinkt sein echter Wert auf den Kartenpreis (Zeile 34).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">•  Deutlich mehr Sparmöglichkeiten stehen auf dem Blatt "Sparhebel" — dort liegt das meiste Geld.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">•  Preise und Konditionen aus deinen Angaben vom 12.08.2026, ergänzt um recherchierte Marktdaten. Vor dem Kauf selbst gegenprüfen.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PSN-Guthabenkarten — wie viele, und zu welchem Preis?</t>
   </si>
   <si>
     <t xml:space="preserve">Grüne Zahlen kommen vom Blatt "Kalkulation".</t>
@@ -210,7 +217,7 @@
     <t xml:space="preserve">Rechnerisch benötigte Karten</t>
   </si>
   <si>
-    <t xml:space="preserve">Eigenanteil geteilt durch 50 €.</t>
+    <t xml:space="preserve">Eigenanteil geteilt durch den Nennwert.</t>
   </si>
   <si>
     <t xml:space="preserve">Karten kaufen (abgerundet)</t>
@@ -288,7 +295,265 @@
     <t xml:space="preserve">Rest zum Eigenanteil</t>
   </si>
   <si>
-    <t xml:space="preserve">Die Spalte "Rest zum Eigenanteil" zeigt, was nach dem Einlösen der Karten noch offen bleibt. Bei 0,00 € ist der Eigenanteil gedeckt.</t>
+    <t xml:space="preserve">Was bringt eine günstigere Bezugsquelle?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Recherchierte Marktpreise für 50 € PSN-Guthaben (Stand August 2026). Alle Zeilen rechnen mit der Kartenzahl aus Variante A.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kaufpreis je 50 €</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rabatt</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Restbetrag bar</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gesamt</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mehrersparnis</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dein aktueller Preis</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Häufige Aktionspreise im Handel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gut erreichbar bei Deal-Portalen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nur bei starken Aktionen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Beworbener Bestpreis — Anbieter genau prüfen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Achtung bei Grauimport-Shops: sehr günstige Codes stammen teils aus fremden Regionen oder aus Rückbuchungen. Ein gesperrter Code oder Account kostet mehr, als die Ersparnis bringt. Halte dich an etablierte Händler mit deutscher Region und Käuferschutz.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Alle Sparhebel im Überblick</t>
+  </si>
+  <si>
+    <t xml:space="preserve">So arbeitest du damit: Trage in der Spalte "Nutzen?" für jeden Hebel Ja, Nein oder Prüfen ein. Nur "Ja" zählt in die gesicherte Ersparnis; "Prüfen" fließt zusätzlich ins Maximalpotenzial.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Stellschrauben — hier drehst du an den Annahmen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bester gefundener Marktpreis der Konsole</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Preisvergleiche listen die Pro deutlich unter der UVP von 899,99 €. Trage den Preis ein, den du wirklich findest.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cashback-Portal — Quote</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Shoop, iGraal &amp; Co. liegen bei 1-5 %. Konsolen sind oft ausgeschlossen — Bedingungen lesen.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kreditkarten-/Payback-Cashback</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Je nach Karte 0,5-2 % auf den Umsatz.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Corporate Benefits / Mitarbeiterrabatt</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Über Arbeitgeberportale oft 3-10 % bei großen Elektronikhändlern.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Newsletter-Gutschein für Neukunden</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Typisch 5-15 €, meist mit Mindestbestellwert.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Punkteaktion auf Guthabenkarten</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Supermärkte fahren regelmäßig 10-20fach-Punkte auf PSN-Karten. Basis ist der Kartenwert.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Preis der günstigsten seriösen PSN-Karte</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Recherchiert: 41-42 € sind bei Deal-Portalen gut erreichbar.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Wert des Disc-Laufwerks der Slim</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UVP des abnehmbaren Laufwerks CFI-ZDD1.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Erwarteter Privatverkaufspreis der Slim</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Was du bei Kleinanzeigen realistisch bekommst.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Die Hebel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hebel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nutzen?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Zählt sicher</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Max. möglich</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Worauf du achten musst</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A — Am Kaufpreis der Konsole selbst sparen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Woanders kaufen statt zur UVP bei PlayStation Direct</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Prüfen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gegenrechnung: Der günstigere Händler spart am Preis, kostet dich aber den 50-€-Eintauschbonus. Nur der Nettovorteil steht hier.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Auf Aktionswoche oder Black Friday warten</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nein</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ALTERNATIVE zum Hebel darüber — nur einer davon kann gelten. Auf "Ja" setzen, wenn du diesen Weg wählst. Trage ein, was du dir vom Warten erwartest.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Refurbished von Sony oder B-Ware statt Neuware</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ALTERNATIVE zu den Hebeln darüber. Mit Herstellergarantie, eventuell leichte Gebrauchsspuren.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bundle kaufen und beiliegendes Spiel weiterverkaufen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ALTERNATIVE zu den Hebeln darüber. Lohnt nur, wenn das Bundle nicht teurer ist als die nackte Konsole.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B — Rabatte, die oben drauf kommen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cashback-Portal vorschalten</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vor dem Kauf über das Portal einsteigen, sonst zählt es nicht. Konsolen sind häufig ausgeschlossen.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kreditkarten- oder Payback-Cashback</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Läuft automatisch über die Zahlungsart, lässt sich meist mit allem kombinieren.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ALTERNATIVE zum Cashback-Portal — beide verlangen einen eigenen Kaufweg. Wenn dein Arbeitgeber ein Portal hat, hier auf "Ja" und Cashback auf "Nein".</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Newsletter-Gutschein als Neukunde</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Einmalig pro Händler, oft mit Mindestbestellwert.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Punkteaktion auf Guthabenkarten mitnehmen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Karten im Supermarkt während einer Punkteaktion kaufen. Punkte anschließend in Prämien oder Cent umwandeln.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Günstigere PSN-Kartenquelle nutzen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dein Preis liegt bei 45,49 €, gut erreichbar sind 41-42 €. Nur seriöse Händler mit deutscher Region.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C — Kosten vermeiden und Zusatzerlöse</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Disc-Laufwerk der Slim behalten statt mitzugeben</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bestätigt: Das abnehmbare Laufwerk CFI-ZDD1 der PS5 Slim passt an die PS5 Pro. Vor dem Eintausch klären, ob es abgegeben werden muss — sonst verschenkst du ein 79,99-€-Teil.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Privatverkauf statt Eintausch, falls er mehr bringt</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Zählt nur, was über Eintauschwert plus Bonus hinausgeht. Bei 372 € Erwartung ist der Eintausch besser.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vorhandenes Zubehör weiternutzen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ja</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DualSense, HDMI-Kabel und Standfuß der Slim passen weiter. Kostet nichts und spart Neukäufe.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nachträgliche Preisgarantie geltend machen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Manche Händler erstatten die Differenz, wenn der Preis binnen 14-30 Tagen fällt. Nach dem Kauf beobachten.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Spiele und Zubehör der Slim separat verkaufen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Discs, Zweitcontroller und Ladestationen bringen einzeln oft mehr als im Paket.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Was dabei herauskommt</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bester Plan bisher (Variante A)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Aus dem Blatt "PSN-Karten" — Stand vor den Hebeln dieser Seite.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gesicherte Zusatzersparnis</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Summe aller Hebel, die du auf "Ja" gesetzt hast.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Zusätzlich möglich, wenn die Prüfungen klappen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Alles, was noch auf "Prüfen" steht.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Endpreis mit gesicherten Hebeln</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Das zahlst du nach heutigem Stand.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Endpreis, wenn alle Hebel greifen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Optimistisch — mehrere Hebel schließen sich in der Praxis gegenseitig aus.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Warum das Best-Case-Ergebnis nicht wörtlich zu nehmen ist: "Woanders kaufen", "Refurbished" und "Auf Aktion warten" beschreiben denselben Kauf auf drei Wegen — du kannst nur einen gehen. Ebenso schließen sich Cashback-Portal und Corporate Benefits meist aus, weil beide einen eigenen Kaufweg verlangen. Setze diese Zeilen bewusst auf "Nein", sobald du dich entschieden hast, dann stimmt die Summe.</t>
   </si>
   <si>
     <t xml:space="preserve">Szenarien im Vergleich</t>
@@ -330,34 +595,52 @@
     <t xml:space="preserve">Eintausch über die Bonus-Aktion abwickeln.</t>
   </si>
   <si>
-    <t xml:space="preserve">5 — Plus PSN-Karten, Variante A</t>
+    <t xml:space="preserve">5 — Plus PSN-Karten zu 45,49 €</t>
   </si>
   <si>
     <t xml:space="preserve">Volle Karten günstig kaufen, Rest normal zahlen.</t>
   </si>
   <si>
-    <t xml:space="preserve">6 — Plus PSN-Karten, Variante B</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Aufrunden — höhere Barkosten, Restguthaben bleibt übrig.</t>
+    <t xml:space="preserve">6 — Plus PSN-Karten, aufgerundet</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Höhere Barkosten, Restguthaben bleibt übrig.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7 — Plus gesicherte Sparhebel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Alle Hebel, die auf "Ja" stehen.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">8 — Best Case, alle Hebel greifen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Optimistisch — siehe Warnung auf dem Blatt "Sparhebel".</t>
   </si>
   <si>
     <t xml:space="preserve">Ergebnis</t>
   </si>
   <si>
-    <t xml:space="preserve">Günstigste Variante (Barkosten)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Kleinster Betrag aus der Tabelle oben.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Gesamtersparnis gegenüber Listenpreis</t>
+    <t xml:space="preserve">Realistisch günstigste Variante</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ohne das optimistische Best-Case-Szenario 8.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ersparnis gegenüber Listenpreis</t>
   </si>
   <si>
     <t xml:space="preserve">Ersparnis in Prozent</t>
   </si>
   <si>
-    <t xml:space="preserve">Empfehlung: Szenario 5. Es hat die niedrigsten echten Barkosten, weil kein Guthaben ungenutzt auf dem PSN-Konto liegen bleibt. Szenario 6 sieht rechnerisch nur dann besser aus, wenn du das Restguthaben ohnehin für Spiele ausgeben würdest.</t>
+    <t xml:space="preserve">Best Case inklusive Szenario 8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nur erreichbar, wenn sich die Hebel nicht gegenseitig ausschließen.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reihenfolge fürs Vorgehen: 1. Klären, ob die Konsole überhaupt mit PSN-Guthaben bezahlbar ist. 2. Preis der Konsole beim günstigsten seriösen Händler gegen das PS-Direct-Paket aus Rabatt und Eintauschbonus rechnen. 3. Vor dem Eintausch das Disc-Laufwerk sichern. 4. Guthabenkarten erst kurz vor dem Kauf und nur bei einer laufenden Aktion holen.</t>
   </si>
 </sst>
 </file>
@@ -371,7 +654,7 @@
     <numFmt numFmtId="167" formatCode="0.00"/>
     <numFmt numFmtId="168" formatCode="0"/>
   </numFmts>
-  <fonts count="14">
+  <fonts count="15">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -469,8 +752,16 @@
       <family val="0"/>
       <charset val="1"/>
     </font>
+    <font>
+      <b val="true"/>
+      <sz val="11"/>
+      <color rgb="FF1F3864"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -499,6 +790,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFE2EFDA"/>
         <bgColor rgb="FFDCE6F1"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFCE4D6"/>
+        <bgColor rgb="FFE2EFDA"/>
       </patternFill>
     </fill>
     <fill>
@@ -577,7 +874,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="56">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -634,6 +931,10 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="166" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -648,6 +949,10 @@
     </xf>
     <xf numFmtId="165" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
@@ -682,11 +987,43 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="6" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="7" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="8" fillId="6" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="8" fillId="7" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="9" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="9" fillId="7" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="8" fillId="7" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="9" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -694,6 +1031,38 @@
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="14" fillId="7" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="7" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="4" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="9" fillId="4" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="11" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="11" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -702,10 +1071,6 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="11" fillId="5" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -718,15 +1083,19 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="5" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="11" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="5" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="8" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -759,7 +1128,7 @@
       <rgbColor rgb="FF7F7F7F"/>
       <rgbColor rgb="FF9999FF"/>
       <rgbColor rgb="FF993366"/>
-      <rgbColor rgb="FFFFFFCC"/>
+      <rgbColor rgb="FFFCE4D6"/>
       <rgbColor rgb="FFDCE6F1"/>
       <rgbColor rgb="FF660066"/>
       <rgbColor rgb="FFFF8080"/>
@@ -982,12 +1351,12 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C41"/>
+  <dimension ref="A1:C42"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="44"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="62"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="74"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1171,7 +1540,7 @@
       <c r="C22" s="4"/>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="8" t="s">
+      <c r="A23" s="14" t="s">
         <v>29</v>
       </c>
     </row>
@@ -1191,143 +1560,154 @@
       <c r="A26" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="B26" s="14" t="n">
+      <c r="B26" s="15" t="n">
         <f aca="false">(B10-B11)/B10</f>
         <v>0.0902</v>
       </c>
+      <c r="C26" s="8" t="s">
+        <v>33</v>
+      </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="15" t="s">
-        <v>33</v>
-      </c>
-      <c r="B27" s="16" t="n">
+      <c r="A27" s="16" t="s">
+        <v>34</v>
+      </c>
+      <c r="B27" s="17" t="n">
         <f aca="false">'PSN-Karten'!B18</f>
         <v>396.91</v>
       </c>
       <c r="C27" s="8" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="6" t="s">
-        <v>35</v>
-      </c>
-      <c r="B28" s="17" t="n">
+        <v>36</v>
+      </c>
+      <c r="B28" s="18" t="n">
         <f aca="false">'PSN-Karten'!B25</f>
         <v>409.41</v>
       </c>
       <c r="C28" s="8" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="6" t="s">
-        <v>37</v>
-      </c>
-      <c r="B29" s="17" t="n">
+        <v>38</v>
+      </c>
+      <c r="B29" s="18" t="n">
         <f aca="false">'PSN-Karten'!B24</f>
         <v>17.01</v>
       </c>
       <c r="C29" s="8" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="3" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B31" s="4"/>
       <c r="C31" s="4"/>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="6" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B32" s="9" t="n">
         <f aca="false">B8+B9</f>
         <v>422</v>
       </c>
       <c r="C32" s="8" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="6" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B33" s="9" t="n">
         <f aca="false">B8+B9+0.01</f>
         <v>422.01</v>
       </c>
       <c r="C33" s="8" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="6" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B34" s="9" t="n">
         <f aca="false">B9/B10*B11</f>
         <v>45.49</v>
       </c>
       <c r="C34" s="8" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="6" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B35" s="9" t="n">
         <f aca="false">B8+B9/B10*B11</f>
         <v>417.49</v>
       </c>
       <c r="C35" s="8" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="3" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B37" s="4"/>
       <c r="C37" s="4"/>
     </row>
-    <row r="38" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A38" s="18" t="s">
-        <v>49</v>
-      </c>
-      <c r="B38" s="18"/>
-      <c r="C38" s="18"/>
-    </row>
-    <row r="39" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A39" s="18" t="s">
+    <row r="38" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A38" s="19" t="s">
         <v>50</v>
       </c>
-      <c r="B39" s="18"/>
-      <c r="C39" s="18"/>
-    </row>
-    <row r="40" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A40" s="18" t="s">
+      <c r="B38" s="19"/>
+      <c r="C38" s="19"/>
+    </row>
+    <row r="39" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A39" s="20" t="s">
         <v>51</v>
       </c>
-      <c r="B40" s="18"/>
-      <c r="C40" s="18"/>
-    </row>
-    <row r="41" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A41" s="18" t="s">
+      <c r="B39" s="20"/>
+      <c r="C39" s="20"/>
+    </row>
+    <row r="40" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A40" s="20" t="s">
         <v>52</v>
       </c>
-      <c r="B41" s="18"/>
-      <c r="C41" s="18"/>
+      <c r="B40" s="20"/>
+      <c r="C40" s="20"/>
+    </row>
+    <row r="41" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A41" s="20" t="s">
+        <v>53</v>
+      </c>
+      <c r="B41" s="20"/>
+      <c r="C41" s="20"/>
+    </row>
+    <row r="42" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A42" s="20" t="s">
+        <v>54</v>
+      </c>
+      <c r="B42" s="20"/>
+      <c r="C42" s="20"/>
     </row>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="5">
     <mergeCell ref="A38:C38"/>
     <mergeCell ref="A39:C39"/>
     <mergeCell ref="A40:C40"/>
     <mergeCell ref="A41:C41"/>
+    <mergeCell ref="A42:C42"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -1344,61 +1724,63 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E44"/>
+  <dimension ref="A1:G54"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="44"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="2" style="0" width="15"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="46"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="B4" s="4"/>
       <c r="C4" s="4"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
-        <v>56</v>
-      </c>
-      <c r="B5" s="17" t="n">
+        <v>58</v>
+      </c>
+      <c r="B5" s="18" t="n">
         <f aca="false">Kalkulation!B20</f>
         <v>432.99</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>57</v>
-      </c>
-      <c r="B6" s="17" t="n">
+        <v>59</v>
+      </c>
+      <c r="B6" s="18" t="n">
         <f aca="false">Kalkulation!B10</f>
         <v>50</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>58</v>
-      </c>
-      <c r="B7" s="17" t="n">
+        <v>60</v>
+      </c>
+      <c r="B7" s="18" t="n">
         <f aca="false">Kalkulation!B11</f>
         <v>45.49</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="B8" s="9" t="n">
         <f aca="false">B6-B7</f>
@@ -1409,45 +1791,45 @@
       <c r="A9" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="B9" s="14" t="n">
+      <c r="B9" s="15" t="n">
         <f aca="false">B8/B6</f>
         <v>0.0902</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="3" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="B11" s="4"/>
       <c r="C11" s="4"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="6" t="s">
-        <v>61</v>
-      </c>
-      <c r="B12" s="19" t="n">
+        <v>63</v>
+      </c>
+      <c r="B12" s="21" t="n">
         <f aca="false">B5/B6</f>
         <v>8.6598</v>
       </c>
       <c r="C12" s="8" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="6" t="s">
-        <v>63</v>
-      </c>
-      <c r="B13" s="20" t="n">
+        <v>65</v>
+      </c>
+      <c r="B13" s="22" t="n">
         <f aca="false">ROUNDDOWN(B5/B6,0)</f>
         <v>8</v>
       </c>
       <c r="C13" s="8" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="6" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="B14" s="9" t="n">
         <f aca="false">B13*B6</f>
@@ -1456,7 +1838,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="6" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="B15" s="9" t="n">
         <f aca="false">B13*B7</f>
@@ -1465,43 +1847,43 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="6" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="B16" s="9" t="n">
         <f aca="false">B5-B14</f>
         <v>32.99</v>
       </c>
       <c r="C16" s="8" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="6" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="B17" s="9" t="n">
         <f aca="false">0</f>
         <v>0</v>
       </c>
       <c r="C17" s="8" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="15" t="s">
-        <v>71</v>
-      </c>
-      <c r="B18" s="21" t="n">
+      <c r="A18" s="16" t="s">
+        <v>73</v>
+      </c>
+      <c r="B18" s="23" t="n">
         <f aca="false">B15+B16</f>
         <v>396.91</v>
       </c>
       <c r="C18" s="8" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="6" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="B19" s="9" t="n">
         <f aca="false">B5-B18</f>
@@ -1510,23 +1892,23 @@
     </row>
     <row r="21" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="3" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="B21" s="4"/>
       <c r="C21" s="4"/>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="6" t="s">
-        <v>75</v>
-      </c>
-      <c r="B22" s="20" t="n">
+        <v>77</v>
+      </c>
+      <c r="B22" s="22" t="n">
         <f aca="false">ROUNDUP(B5/B6,0)</f>
         <v>9</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="6" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="B23" s="9" t="n">
         <f aca="false">B22*B6</f>
@@ -1535,31 +1917,31 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="6" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B24" s="9" t="n">
         <f aca="false">B23-B5</f>
         <v>17.01</v>
       </c>
       <c r="C24" s="8" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="22" t="s">
-        <v>78</v>
+      <c r="A25" s="24" t="s">
+        <v>80</v>
       </c>
       <c r="B25" s="11" t="n">
         <f aca="false">B22*B7</f>
         <v>409.41</v>
       </c>
       <c r="C25" s="8" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="6" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="B26" s="9" t="n">
         <f aca="false">B5-B25</f>
@@ -1568,304 +1950,489 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="6" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B27" s="9" t="n">
         <f aca="false">B25-B24</f>
         <v>392.4</v>
       </c>
       <c r="C27" s="8" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="3" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="B29" s="4"/>
       <c r="C29" s="4"/>
+      <c r="D29" s="4"/>
+      <c r="E29" s="4"/>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="23" t="s">
-        <v>83</v>
-      </c>
-      <c r="B30" s="23" t="s">
-        <v>84</v>
-      </c>
-      <c r="C30" s="23" t="s">
+      <c r="A30" s="25" t="s">
         <v>85</v>
       </c>
-      <c r="D30" s="23" t="s">
+      <c r="B30" s="25" t="s">
         <v>86</v>
       </c>
-      <c r="E30" s="23" t="s">
+      <c r="C30" s="25" t="s">
         <v>87</v>
       </c>
+      <c r="D30" s="25" t="s">
+        <v>88</v>
+      </c>
+      <c r="E30" s="25" t="s">
+        <v>89</v>
+      </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="24" t="n">
+      <c r="A31" s="26" t="n">
         <v>1</v>
       </c>
-      <c r="B31" s="25" t="n">
+      <c r="B31" s="27" t="n">
         <f aca="false">A31*$B$6</f>
         <v>50</v>
       </c>
-      <c r="C31" s="25" t="n">
+      <c r="C31" s="27" t="n">
         <f aca="false">A31*$B$7</f>
         <v>45.49</v>
       </c>
-      <c r="D31" s="25" t="n">
+      <c r="D31" s="27" t="n">
         <f aca="false">A31*($B$6-$B$7)</f>
         <v>4.51</v>
       </c>
-      <c r="E31" s="25" t="n">
+      <c r="E31" s="27" t="n">
         <f aca="false">MAX(0,$B$5-B31)</f>
         <v>382.99</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="26" t="n">
+      <c r="A32" s="28" t="n">
         <v>2</v>
       </c>
-      <c r="B32" s="27" t="n">
+      <c r="B32" s="29" t="n">
         <f aca="false">A32*$B$6</f>
         <v>100</v>
       </c>
-      <c r="C32" s="27" t="n">
+      <c r="C32" s="29" t="n">
         <f aca="false">A32*$B$7</f>
         <v>90.98</v>
       </c>
-      <c r="D32" s="27" t="n">
+      <c r="D32" s="29" t="n">
         <f aca="false">A32*($B$6-$B$7)</f>
         <v>9.02</v>
       </c>
-      <c r="E32" s="27" t="n">
+      <c r="E32" s="29" t="n">
         <f aca="false">MAX(0,$B$5-B32)</f>
         <v>332.99</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="24" t="n">
+      <c r="A33" s="26" t="n">
         <v>3</v>
       </c>
-      <c r="B33" s="25" t="n">
+      <c r="B33" s="27" t="n">
         <f aca="false">A33*$B$6</f>
         <v>150</v>
       </c>
-      <c r="C33" s="25" t="n">
+      <c r="C33" s="27" t="n">
         <f aca="false">A33*$B$7</f>
         <v>136.47</v>
       </c>
-      <c r="D33" s="25" t="n">
+      <c r="D33" s="27" t="n">
         <f aca="false">A33*($B$6-$B$7)</f>
         <v>13.53</v>
       </c>
-      <c r="E33" s="25" t="n">
+      <c r="E33" s="27" t="n">
         <f aca="false">MAX(0,$B$5-B33)</f>
         <v>282.99</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="26" t="n">
+      <c r="A34" s="28" t="n">
         <v>4</v>
       </c>
-      <c r="B34" s="27" t="n">
+      <c r="B34" s="29" t="n">
         <f aca="false">A34*$B$6</f>
         <v>200</v>
       </c>
-      <c r="C34" s="27" t="n">
+      <c r="C34" s="29" t="n">
         <f aca="false">A34*$B$7</f>
         <v>181.96</v>
       </c>
-      <c r="D34" s="27" t="n">
+      <c r="D34" s="29" t="n">
         <f aca="false">A34*($B$6-$B$7)</f>
         <v>18.04</v>
       </c>
-      <c r="E34" s="27" t="n">
+      <c r="E34" s="29" t="n">
         <f aca="false">MAX(0,$B$5-B34)</f>
         <v>232.99</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="24" t="n">
+      <c r="A35" s="26" t="n">
         <v>5</v>
       </c>
-      <c r="B35" s="25" t="n">
+      <c r="B35" s="27" t="n">
         <f aca="false">A35*$B$6</f>
         <v>250</v>
       </c>
-      <c r="C35" s="25" t="n">
+      <c r="C35" s="27" t="n">
         <f aca="false">A35*$B$7</f>
         <v>227.45</v>
       </c>
-      <c r="D35" s="25" t="n">
+      <c r="D35" s="27" t="n">
         <f aca="false">A35*($B$6-$B$7)</f>
         <v>22.55</v>
       </c>
-      <c r="E35" s="25" t="n">
+      <c r="E35" s="27" t="n">
         <f aca="false">MAX(0,$B$5-B35)</f>
         <v>182.99</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="26" t="n">
+      <c r="A36" s="28" t="n">
         <v>6</v>
       </c>
-      <c r="B36" s="27" t="n">
+      <c r="B36" s="29" t="n">
         <f aca="false">A36*$B$6</f>
         <v>300</v>
       </c>
-      <c r="C36" s="27" t="n">
+      <c r="C36" s="29" t="n">
         <f aca="false">A36*$B$7</f>
         <v>272.94</v>
       </c>
-      <c r="D36" s="27" t="n">
+      <c r="D36" s="29" t="n">
         <f aca="false">A36*($B$6-$B$7)</f>
         <v>27.06</v>
       </c>
-      <c r="E36" s="27" t="n">
+      <c r="E36" s="29" t="n">
         <f aca="false">MAX(0,$B$5-B36)</f>
         <v>132.99</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="24" t="n">
+      <c r="A37" s="26" t="n">
         <v>7</v>
       </c>
-      <c r="B37" s="25" t="n">
+      <c r="B37" s="27" t="n">
         <f aca="false">A37*$B$6</f>
         <v>350</v>
       </c>
-      <c r="C37" s="25" t="n">
+      <c r="C37" s="27" t="n">
         <f aca="false">A37*$B$7</f>
         <v>318.43</v>
       </c>
-      <c r="D37" s="25" t="n">
+      <c r="D37" s="27" t="n">
         <f aca="false">A37*($B$6-$B$7)</f>
         <v>31.57</v>
       </c>
-      <c r="E37" s="25" t="n">
+      <c r="E37" s="27" t="n">
         <f aca="false">MAX(0,$B$5-B37)</f>
         <v>82.99</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="26" t="n">
+      <c r="A38" s="28" t="n">
         <v>8</v>
       </c>
-      <c r="B38" s="27" t="n">
+      <c r="B38" s="29" t="n">
         <f aca="false">A38*$B$6</f>
         <v>400</v>
       </c>
-      <c r="C38" s="27" t="n">
+      <c r="C38" s="29" t="n">
         <f aca="false">A38*$B$7</f>
         <v>363.92</v>
       </c>
-      <c r="D38" s="27" t="n">
+      <c r="D38" s="29" t="n">
         <f aca="false">A38*($B$6-$B$7)</f>
         <v>36.08</v>
       </c>
-      <c r="E38" s="27" t="n">
+      <c r="E38" s="29" t="n">
         <f aca="false">MAX(0,$B$5-B38)</f>
         <v>32.99</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="24" t="n">
+      <c r="A39" s="26" t="n">
         <v>9</v>
       </c>
-      <c r="B39" s="25" t="n">
+      <c r="B39" s="27" t="n">
         <f aca="false">A39*$B$6</f>
         <v>450</v>
       </c>
-      <c r="C39" s="25" t="n">
+      <c r="C39" s="27" t="n">
         <f aca="false">A39*$B$7</f>
         <v>409.41</v>
       </c>
-      <c r="D39" s="25" t="n">
+      <c r="D39" s="27" t="n">
         <f aca="false">A39*($B$6-$B$7)</f>
         <v>40.59</v>
       </c>
-      <c r="E39" s="25" t="n">
+      <c r="E39" s="27" t="n">
         <f aca="false">MAX(0,$B$5-B39)</f>
         <v>0</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="26" t="n">
+      <c r="A40" s="28" t="n">
         <v>10</v>
       </c>
-      <c r="B40" s="27" t="n">
+      <c r="B40" s="29" t="n">
         <f aca="false">A40*$B$6</f>
         <v>500</v>
       </c>
-      <c r="C40" s="27" t="n">
+      <c r="C40" s="29" t="n">
         <f aca="false">A40*$B$7</f>
         <v>454.9</v>
       </c>
-      <c r="D40" s="27" t="n">
+      <c r="D40" s="29" t="n">
         <f aca="false">A40*($B$6-$B$7)</f>
         <v>45.1</v>
       </c>
-      <c r="E40" s="27" t="n">
+      <c r="E40" s="29" t="n">
         <f aca="false">MAX(0,$B$5-B40)</f>
         <v>0</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="24" t="n">
+      <c r="A41" s="26" t="n">
         <v>11</v>
       </c>
-      <c r="B41" s="25" t="n">
+      <c r="B41" s="27" t="n">
         <f aca="false">A41*$B$6</f>
         <v>550</v>
       </c>
-      <c r="C41" s="25" t="n">
+      <c r="C41" s="27" t="n">
         <f aca="false">A41*$B$7</f>
         <v>500.39</v>
       </c>
-      <c r="D41" s="25" t="n">
+      <c r="D41" s="27" t="n">
         <f aca="false">A41*($B$6-$B$7)</f>
         <v>49.61</v>
       </c>
-      <c r="E41" s="25" t="n">
+      <c r="E41" s="27" t="n">
         <f aca="false">MAX(0,$B$5-B41)</f>
         <v>0</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="26" t="n">
+      <c r="A42" s="28" t="n">
         <v>12</v>
       </c>
-      <c r="B42" s="27" t="n">
+      <c r="B42" s="29" t="n">
         <f aca="false">A42*$B$6</f>
         <v>600</v>
       </c>
-      <c r="C42" s="27" t="n">
+      <c r="C42" s="29" t="n">
         <f aca="false">A42*$B$7</f>
         <v>545.88</v>
       </c>
-      <c r="D42" s="27" t="n">
+      <c r="D42" s="29" t="n">
         <f aca="false">A42*($B$6-$B$7)</f>
         <v>54.12</v>
       </c>
-      <c r="E42" s="27" t="n">
+      <c r="E42" s="29" t="n">
         <f aca="false">MAX(0,$B$5-B42)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="44" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A44" s="18" t="s">
-        <v>88</v>
-      </c>
-      <c r="B44" s="18"/>
-      <c r="C44" s="18"/>
-      <c r="D44" s="18"/>
-      <c r="E44" s="18"/>
+    <row r="45" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A45" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="B45" s="4"/>
+      <c r="C45" s="4"/>
+      <c r="D45" s="4"/>
+      <c r="E45" s="4"/>
+      <c r="F45" s="4"/>
+    </row>
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A46" s="30" t="s">
+        <v>91</v>
+      </c>
+      <c r="B46" s="30"/>
+      <c r="C46" s="30"/>
+      <c r="D46" s="30"/>
+      <c r="E46" s="30"/>
+      <c r="F46" s="30"/>
+    </row>
+    <row r="47" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A47" s="31" t="s">
+        <v>92</v>
+      </c>
+      <c r="B47" s="31" t="s">
+        <v>93</v>
+      </c>
+      <c r="C47" s="31" t="s">
+        <v>68</v>
+      </c>
+      <c r="D47" s="31" t="s">
+        <v>94</v>
+      </c>
+      <c r="E47" s="31" t="s">
+        <v>95</v>
+      </c>
+      <c r="F47" s="31" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A48" s="32" t="n">
+        <v>45.49</v>
+      </c>
+      <c r="B48" s="33" t="n">
+        <f aca="false">($B$6-A48)/$B$6</f>
+        <v>0.0902</v>
+      </c>
+      <c r="C48" s="27" t="n">
+        <f aca="false">$B$13*A48</f>
+        <v>363.92</v>
+      </c>
+      <c r="D48" s="27" t="n">
+        <f aca="false">$B$16</f>
+        <v>32.99</v>
+      </c>
+      <c r="E48" s="27" t="n">
+        <f aca="false">C48+D48</f>
+        <v>396.91</v>
+      </c>
+      <c r="F48" s="27" t="n">
+        <f aca="false">$B$18-E48</f>
+        <v>0</v>
+      </c>
+      <c r="G48" s="14" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A49" s="34" t="n">
+        <v>43.99</v>
+      </c>
+      <c r="B49" s="35" t="n">
+        <f aca="false">($B$6-A49)/$B$6</f>
+        <v>0.1202</v>
+      </c>
+      <c r="C49" s="29" t="n">
+        <f aca="false">$B$13*A49</f>
+        <v>351.92</v>
+      </c>
+      <c r="D49" s="29" t="n">
+        <f aca="false">$B$16</f>
+        <v>32.99</v>
+      </c>
+      <c r="E49" s="29" t="n">
+        <f aca="false">C49+D49</f>
+        <v>384.91</v>
+      </c>
+      <c r="F49" s="29" t="n">
+        <f aca="false">$B$18-E49</f>
+        <v>12</v>
+      </c>
+      <c r="G49" s="14" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A50" s="32" t="n">
+        <v>41.99</v>
+      </c>
+      <c r="B50" s="33" t="n">
+        <f aca="false">($B$6-A50)/$B$6</f>
+        <v>0.1602</v>
+      </c>
+      <c r="C50" s="27" t="n">
+        <f aca="false">$B$13*A50</f>
+        <v>335.92</v>
+      </c>
+      <c r="D50" s="27" t="n">
+        <f aca="false">$B$16</f>
+        <v>32.99</v>
+      </c>
+      <c r="E50" s="27" t="n">
+        <f aca="false">C50+D50</f>
+        <v>368.91</v>
+      </c>
+      <c r="F50" s="27" t="n">
+        <f aca="false">$B$18-E50</f>
+        <v>28</v>
+      </c>
+      <c r="G50" s="14" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A51" s="34" t="n">
+        <v>39.99</v>
+      </c>
+      <c r="B51" s="35" t="n">
+        <f aca="false">($B$6-A51)/$B$6</f>
+        <v>0.2002</v>
+      </c>
+      <c r="C51" s="29" t="n">
+        <f aca="false">$B$13*A51</f>
+        <v>319.92</v>
+      </c>
+      <c r="D51" s="29" t="n">
+        <f aca="false">$B$16</f>
+        <v>32.99</v>
+      </c>
+      <c r="E51" s="29" t="n">
+        <f aca="false">C51+D51</f>
+        <v>352.91</v>
+      </c>
+      <c r="F51" s="29" t="n">
+        <f aca="false">$B$18-E51</f>
+        <v>44</v>
+      </c>
+      <c r="G51" s="14" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A52" s="32" t="n">
+        <v>37.5</v>
+      </c>
+      <c r="B52" s="33" t="n">
+        <f aca="false">($B$6-A52)/$B$6</f>
+        <v>0.25</v>
+      </c>
+      <c r="C52" s="27" t="n">
+        <f aca="false">$B$13*A52</f>
+        <v>300</v>
+      </c>
+      <c r="D52" s="27" t="n">
+        <f aca="false">$B$16</f>
+        <v>32.99</v>
+      </c>
+      <c r="E52" s="27" t="n">
+        <f aca="false">C52+D52</f>
+        <v>332.99</v>
+      </c>
+      <c r="F52" s="27" t="n">
+        <f aca="false">$B$18-E52</f>
+        <v>63.92</v>
+      </c>
+      <c r="G52" s="14" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="54" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A54" s="19" t="s">
+        <v>102</v>
+      </c>
+      <c r="B54" s="19"/>
+      <c r="C54" s="19"/>
+      <c r="D54" s="19"/>
+      <c r="E54" s="19"/>
+      <c r="F54" s="19"/>
+      <c r="G54" s="19"/>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A44:E44"/>
+  <mergeCells count="2">
+    <mergeCell ref="A46:F46"/>
+    <mergeCell ref="A54:G54"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -1882,184 +2449,868 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D17"/>
+  <dimension ref="A1:F43"/>
+  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="48"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="76"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="36" t="s">
+        <v>104</v>
+      </c>
+      <c r="B2" s="36"/>
+      <c r="C2" s="36"/>
+      <c r="D2" s="36"/>
+      <c r="E2" s="36"/>
+      <c r="F2" s="36"/>
+    </row>
+    <row r="4" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="3" t="s">
+        <v>105</v>
+      </c>
+      <c r="B4" s="4"/>
+      <c r="C4" s="4"/>
+      <c r="D4" s="4"/>
+      <c r="E4" s="4"/>
+      <c r="F4" s="4"/>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="B5" s="7" t="n">
+        <v>798.9</v>
+      </c>
+      <c r="F5" s="8" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="6" t="s">
+        <v>108</v>
+      </c>
+      <c r="B6" s="37" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="F6" s="8" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="6" t="s">
+        <v>110</v>
+      </c>
+      <c r="B7" s="37" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="F7" s="8" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="6" t="s">
+        <v>112</v>
+      </c>
+      <c r="B8" s="37" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="F8" s="8" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="6" t="s">
+        <v>114</v>
+      </c>
+      <c r="B9" s="7" t="n">
+        <v>10</v>
+      </c>
+      <c r="F9" s="8" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="6" t="s">
+        <v>116</v>
+      </c>
+      <c r="B10" s="37" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="F10" s="8" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="6" t="s">
+        <v>118</v>
+      </c>
+      <c r="B11" s="7" t="n">
+        <v>41.99</v>
+      </c>
+      <c r="F11" s="8" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="6" t="s">
+        <v>120</v>
+      </c>
+      <c r="B12" s="7" t="n">
+        <v>79.99</v>
+      </c>
+      <c r="F12" s="8" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="6" t="s">
+        <v>122</v>
+      </c>
+      <c r="B13" s="7" t="n">
+        <v>372</v>
+      </c>
+      <c r="F13" s="8" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="B15" s="4"/>
+      <c r="C15" s="4"/>
+      <c r="D15" s="4"/>
+      <c r="E15" s="4"/>
+      <c r="F15" s="4"/>
+    </row>
+    <row r="16" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="38" t="s">
+        <v>125</v>
+      </c>
+      <c r="B16" s="38" t="s">
+        <v>88</v>
+      </c>
+      <c r="C16" s="38" t="s">
+        <v>126</v>
+      </c>
+      <c r="D16" s="38" t="s">
+        <v>127</v>
+      </c>
+      <c r="E16" s="38" t="s">
+        <v>128</v>
+      </c>
+      <c r="F16" s="38" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="39" t="s">
+        <v>130</v>
+      </c>
+      <c r="B17" s="40"/>
+      <c r="C17" s="40"/>
+      <c r="D17" s="40"/>
+      <c r="E17" s="40"/>
+      <c r="F17" s="40"/>
+    </row>
+    <row r="18" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="41" t="s">
+        <v>131</v>
+      </c>
+      <c r="B18" s="27" t="n">
+        <f aca="false">MAX(0,Kalkulation!B16-$B$5-Kalkulation!B9)</f>
+        <v>6.09000000000003</v>
+      </c>
+      <c r="C18" s="42" t="s">
+        <v>132</v>
+      </c>
+      <c r="D18" s="27" t="n">
+        <f aca="false">IF(C18="Ja",B18,0)</f>
+        <v>0</v>
+      </c>
+      <c r="E18" s="27" t="n">
+        <f aca="false">IF(OR(C18="Ja",C18="Prüfen"),B18,0)</f>
+        <v>6.09000000000003</v>
+      </c>
+      <c r="F18" s="43" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="41" t="s">
+        <v>134</v>
+      </c>
+      <c r="B19" s="44" t="n">
+        <v>50</v>
+      </c>
+      <c r="C19" s="42" t="s">
+        <v>135</v>
+      </c>
+      <c r="D19" s="27" t="n">
+        <f aca="false">IF(C19="Ja",B19,0)</f>
+        <v>0</v>
+      </c>
+      <c r="E19" s="27" t="n">
+        <f aca="false">IF(OR(C19="Ja",C19="Prüfen"),B19,0)</f>
+        <v>0</v>
+      </c>
+      <c r="F19" s="43" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="41" t="s">
+        <v>137</v>
+      </c>
+      <c r="B20" s="44" t="n">
+        <v>90</v>
+      </c>
+      <c r="C20" s="42" t="s">
+        <v>135</v>
+      </c>
+      <c r="D20" s="27" t="n">
+        <f aca="false">IF(C20="Ja",B20,0)</f>
+        <v>0</v>
+      </c>
+      <c r="E20" s="27" t="n">
+        <f aca="false">IF(OR(C20="Ja",C20="Prüfen"),B20,0)</f>
+        <v>0</v>
+      </c>
+      <c r="F20" s="43" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="41" t="s">
+        <v>139</v>
+      </c>
+      <c r="B21" s="44" t="n">
+        <v>30</v>
+      </c>
+      <c r="C21" s="42" t="s">
+        <v>135</v>
+      </c>
+      <c r="D21" s="27" t="n">
+        <f aca="false">IF(C21="Ja",B21,0)</f>
+        <v>0</v>
+      </c>
+      <c r="E21" s="27" t="n">
+        <f aca="false">IF(OR(C21="Ja",C21="Prüfen"),B21,0)</f>
+        <v>0</v>
+      </c>
+      <c r="F21" s="43" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="39" t="s">
+        <v>141</v>
+      </c>
+      <c r="B22" s="40"/>
+      <c r="C22" s="40"/>
+      <c r="D22" s="40"/>
+      <c r="E22" s="40"/>
+      <c r="F22" s="40"/>
+    </row>
+    <row r="23" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="41" t="s">
+        <v>142</v>
+      </c>
+      <c r="B23" s="27" t="n">
+        <f aca="false">Kalkulation!B16*$B$6</f>
+        <v>25.6497</v>
+      </c>
+      <c r="C23" s="42" t="s">
+        <v>132</v>
+      </c>
+      <c r="D23" s="27" t="n">
+        <f aca="false">IF(C23="Ja",B23,0)</f>
+        <v>0</v>
+      </c>
+      <c r="E23" s="27" t="n">
+        <f aca="false">IF(OR(C23="Ja",C23="Prüfen"),B23,0)</f>
+        <v>25.6497</v>
+      </c>
+      <c r="F23" s="43" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="41" t="s">
+        <v>144</v>
+      </c>
+      <c r="B24" s="27" t="n">
+        <f aca="false">Kalkulation!B16*$B$7</f>
+        <v>8.5499</v>
+      </c>
+      <c r="C24" s="42" t="s">
+        <v>132</v>
+      </c>
+      <c r="D24" s="27" t="n">
+        <f aca="false">IF(C24="Ja",B24,0)</f>
+        <v>0</v>
+      </c>
+      <c r="E24" s="27" t="n">
+        <f aca="false">IF(OR(C24="Ja",C24="Prüfen"),B24,0)</f>
+        <v>8.5499</v>
+      </c>
+      <c r="F24" s="43" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="41" t="s">
+        <v>112</v>
+      </c>
+      <c r="B25" s="27" t="n">
+        <f aca="false">Kalkulation!B16*$B$8</f>
+        <v>25.6497</v>
+      </c>
+      <c r="C25" s="42" t="s">
+        <v>135</v>
+      </c>
+      <c r="D25" s="27" t="n">
+        <f aca="false">IF(C25="Ja",B25,0)</f>
+        <v>0</v>
+      </c>
+      <c r="E25" s="27" t="n">
+        <f aca="false">IF(OR(C25="Ja",C25="Prüfen"),B25,0)</f>
+        <v>0</v>
+      </c>
+      <c r="F25" s="43" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="41" t="s">
+        <v>147</v>
+      </c>
+      <c r="B26" s="27" t="n">
+        <f aca="false">$B$9</f>
+        <v>10</v>
+      </c>
+      <c r="C26" s="42" t="s">
+        <v>132</v>
+      </c>
+      <c r="D26" s="27" t="n">
+        <f aca="false">IF(C26="Ja",B26,0)</f>
+        <v>0</v>
+      </c>
+      <c r="E26" s="27" t="n">
+        <f aca="false">IF(OR(C26="Ja",C26="Prüfen"),B26,0)</f>
+        <v>10</v>
+      </c>
+      <c r="F26" s="43" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="41" t="s">
+        <v>149</v>
+      </c>
+      <c r="B27" s="27" t="n">
+        <f aca="false">'PSN-Karten'!B14*$B$10</f>
+        <v>20</v>
+      </c>
+      <c r="C27" s="42" t="s">
+        <v>132</v>
+      </c>
+      <c r="D27" s="27" t="n">
+        <f aca="false">IF(C27="Ja",B27,0)</f>
+        <v>0</v>
+      </c>
+      <c r="E27" s="27" t="n">
+        <f aca="false">IF(OR(C27="Ja",C27="Prüfen"),B27,0)</f>
+        <v>20</v>
+      </c>
+      <c r="F27" s="43" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="41" t="s">
+        <v>151</v>
+      </c>
+      <c r="B28" s="27" t="n">
+        <f aca="false">'PSN-Karten'!B13*('PSN-Karten'!B7-$B$11)</f>
+        <v>28</v>
+      </c>
+      <c r="C28" s="42" t="s">
+        <v>132</v>
+      </c>
+      <c r="D28" s="27" t="n">
+        <f aca="false">IF(C28="Ja",B28,0)</f>
+        <v>0</v>
+      </c>
+      <c r="E28" s="27" t="n">
+        <f aca="false">IF(OR(C28="Ja",C28="Prüfen"),B28,0)</f>
+        <v>28</v>
+      </c>
+      <c r="F28" s="43" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="39" t="s">
+        <v>153</v>
+      </c>
+      <c r="B29" s="40"/>
+      <c r="C29" s="40"/>
+      <c r="D29" s="40"/>
+      <c r="E29" s="40"/>
+      <c r="F29" s="40"/>
+    </row>
+    <row r="30" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A30" s="41" t="s">
+        <v>154</v>
+      </c>
+      <c r="B30" s="27" t="n">
+        <f aca="false">$B$12</f>
+        <v>79.99</v>
+      </c>
+      <c r="C30" s="42" t="s">
+        <v>132</v>
+      </c>
+      <c r="D30" s="27" t="n">
+        <f aca="false">IF(C30="Ja",B30,0)</f>
+        <v>0</v>
+      </c>
+      <c r="E30" s="27" t="n">
+        <f aca="false">IF(OR(C30="Ja",C30="Prüfen"),B30,0)</f>
+        <v>79.99</v>
+      </c>
+      <c r="F30" s="43" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A31" s="41" t="s">
+        <v>156</v>
+      </c>
+      <c r="B31" s="27" t="n">
+        <f aca="false">MAX(0,$B$13-Kalkulation!B8-Kalkulation!B9)</f>
+        <v>0</v>
+      </c>
+      <c r="C31" s="42" t="s">
+        <v>132</v>
+      </c>
+      <c r="D31" s="27" t="n">
+        <f aca="false">IF(C31="Ja",B31,0)</f>
+        <v>0</v>
+      </c>
+      <c r="E31" s="27" t="n">
+        <f aca="false">IF(OR(C31="Ja",C31="Prüfen"),B31,0)</f>
+        <v>0</v>
+      </c>
+      <c r="F31" s="43" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A32" s="41" t="s">
+        <v>158</v>
+      </c>
+      <c r="B32" s="44" t="n">
+        <v>0</v>
+      </c>
+      <c r="C32" s="42" t="s">
+        <v>159</v>
+      </c>
+      <c r="D32" s="27" t="n">
+        <f aca="false">IF(C32="Ja",B32,0)</f>
+        <v>0</v>
+      </c>
+      <c r="E32" s="27" t="n">
+        <f aca="false">IF(OR(C32="Ja",C32="Prüfen"),B32,0)</f>
+        <v>0</v>
+      </c>
+      <c r="F32" s="43" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A33" s="41" t="s">
+        <v>161</v>
+      </c>
+      <c r="B33" s="44" t="n">
+        <v>0</v>
+      </c>
+      <c r="C33" s="42" t="s">
+        <v>132</v>
+      </c>
+      <c r="D33" s="27" t="n">
+        <f aca="false">IF(C33="Ja",B33,0)</f>
+        <v>0</v>
+      </c>
+      <c r="E33" s="27" t="n">
+        <f aca="false">IF(OR(C33="Ja",C33="Prüfen"),B33,0)</f>
+        <v>0</v>
+      </c>
+      <c r="F33" s="43" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A34" s="41" t="s">
+        <v>163</v>
+      </c>
+      <c r="B34" s="44" t="n">
+        <v>0</v>
+      </c>
+      <c r="C34" s="42" t="s">
+        <v>132</v>
+      </c>
+      <c r="D34" s="27" t="n">
+        <f aca="false">IF(C34="Ja",B34,0)</f>
+        <v>0</v>
+      </c>
+      <c r="E34" s="27" t="n">
+        <f aca="false">IF(OR(C34="Ja",C34="Prüfen"),B34,0)</f>
+        <v>0</v>
+      </c>
+      <c r="F34" s="43" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A36" s="3" t="s">
+        <v>165</v>
+      </c>
+      <c r="B36" s="4"/>
+      <c r="C36" s="4"/>
+      <c r="D36" s="4"/>
+      <c r="E36" s="4"/>
+      <c r="F36" s="4"/>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="6" t="s">
+        <v>166</v>
+      </c>
+      <c r="B37" s="18" t="n">
+        <f aca="false">'PSN-Karten'!B18</f>
+        <v>396.91</v>
+      </c>
+      <c r="F37" s="8" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="6" t="s">
+        <v>168</v>
+      </c>
+      <c r="B38" s="9" t="n">
+        <f aca="false">SUM(D18:D34)</f>
+        <v>0</v>
+      </c>
+      <c r="F38" s="8" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="6" t="s">
+        <v>170</v>
+      </c>
+      <c r="B39" s="9" t="n">
+        <f aca="false">SUM(E18:E34)-SUM(D18:D34)</f>
+        <v>178.2796</v>
+      </c>
+      <c r="F39" s="8" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="16" t="s">
+        <v>172</v>
+      </c>
+      <c r="B40" s="45" t="n">
+        <f aca="false">MAX(0,'PSN-Karten'!B18-SUM(D18:D34))</f>
+        <v>396.91</v>
+      </c>
+      <c r="F40" s="8" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="24" t="s">
+        <v>174</v>
+      </c>
+      <c r="B41" s="46" t="n">
+        <f aca="false">MAX(0,'PSN-Karten'!B18-SUM(E18:E34))</f>
+        <v>218.6304</v>
+      </c>
+      <c r="F41" s="8" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A43" s="19" t="s">
+        <v>176</v>
+      </c>
+      <c r="B43" s="19"/>
+      <c r="C43" s="19"/>
+      <c r="D43" s="19"/>
+      <c r="E43" s="19"/>
+      <c r="F43" s="19"/>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A43:F43"/>
+  </mergeCells>
+  <dataValidations count="1">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="C18:C34" type="list">
+      <formula1>"Ja,Nein,Prüfen"</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+  </dataValidations>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:D20"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="52"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="16"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="54"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="60"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>89</v>
+        <v>177</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>90</v>
+        <v>178</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="28" t="s">
-        <v>91</v>
-      </c>
-      <c r="B4" s="28" t="s">
-        <v>92</v>
-      </c>
-      <c r="C4" s="28" t="s">
-        <v>86</v>
-      </c>
-      <c r="D4" s="28" t="s">
-        <v>93</v>
+      <c r="A4" s="38" t="s">
+        <v>179</v>
+      </c>
+      <c r="B4" s="38" t="s">
+        <v>180</v>
+      </c>
+      <c r="C4" s="38" t="s">
+        <v>88</v>
+      </c>
+      <c r="D4" s="38" t="s">
+        <v>181</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="29" t="s">
-        <v>94</v>
-      </c>
-      <c r="B5" s="30" t="n">
+      <c r="A5" s="47" t="s">
+        <v>182</v>
+      </c>
+      <c r="B5" s="48" t="n">
         <f aca="false">Kalkulation!B6</f>
         <v>899.99</v>
       </c>
-      <c r="C5" s="25" t="n">
+      <c r="C5" s="27" t="n">
         <f aca="false">$B$5-B5</f>
         <v>0</v>
       </c>
-      <c r="D5" s="31" t="s">
-        <v>95</v>
+      <c r="D5" s="43" t="s">
+        <v>183</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="29" t="s">
-        <v>96</v>
-      </c>
-      <c r="B6" s="30" t="n">
+      <c r="A6" s="47" t="s">
+        <v>184</v>
+      </c>
+      <c r="B6" s="48" t="n">
         <f aca="false">Kalkulation!B16</f>
         <v>854.99</v>
       </c>
-      <c r="C6" s="25" t="n">
+      <c r="C6" s="27" t="n">
         <f aca="false">$B$5-B6</f>
         <v>45</v>
       </c>
-      <c r="D6" s="31" t="s">
-        <v>97</v>
+      <c r="D6" s="43" t="s">
+        <v>185</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="29" t="s">
-        <v>98</v>
-      </c>
-      <c r="B7" s="30" t="n">
+      <c r="A7" s="47" t="s">
+        <v>186</v>
+      </c>
+      <c r="B7" s="48" t="n">
         <f aca="false">Kalkulation!B18</f>
         <v>482.99</v>
       </c>
-      <c r="C7" s="25" t="n">
+      <c r="C7" s="27" t="n">
         <f aca="false">$B$5-B7</f>
         <v>417</v>
       </c>
-      <c r="D7" s="31" t="s">
-        <v>99</v>
+      <c r="D7" s="43" t="s">
+        <v>187</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="29" t="s">
-        <v>100</v>
-      </c>
-      <c r="B8" s="30" t="n">
+      <c r="A8" s="47" t="s">
+        <v>188</v>
+      </c>
+      <c r="B8" s="48" t="n">
         <f aca="false">Kalkulation!B20</f>
         <v>432.99</v>
       </c>
-      <c r="C8" s="25" t="n">
+      <c r="C8" s="27" t="n">
         <f aca="false">$B$5-B8</f>
         <v>467</v>
       </c>
-      <c r="D8" s="31" t="s">
-        <v>101</v>
+      <c r="D8" s="43" t="s">
+        <v>189</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="32" t="s">
-        <v>102</v>
-      </c>
-      <c r="B9" s="33" t="n">
+      <c r="A9" s="47" t="s">
+        <v>190</v>
+      </c>
+      <c r="B9" s="48" t="n">
         <f aca="false">'PSN-Karten'!B18</f>
         <v>396.91</v>
       </c>
-      <c r="C9" s="34" t="n">
+      <c r="C9" s="27" t="n">
         <f aca="false">$B$5-B9</f>
         <v>503.08</v>
       </c>
-      <c r="D9" s="35" t="s">
-        <v>103</v>
+      <c r="D9" s="43" t="s">
+        <v>191</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="29" t="s">
-        <v>104</v>
-      </c>
-      <c r="B10" s="30" t="n">
+      <c r="A10" s="47" t="s">
+        <v>192</v>
+      </c>
+      <c r="B10" s="48" t="n">
         <f aca="false">'PSN-Karten'!B25</f>
         <v>409.41</v>
       </c>
-      <c r="C10" s="25" t="n">
+      <c r="C10" s="27" t="n">
         <f aca="false">$B$5-B10</f>
         <v>490.58</v>
       </c>
-      <c r="D10" s="31" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="3" t="s">
-        <v>106</v>
-      </c>
-      <c r="B12" s="4"/>
-      <c r="C12" s="4"/>
-      <c r="D12" s="4"/>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="22" t="s">
-        <v>107</v>
-      </c>
-      <c r="B13" s="36" t="n">
-        <f aca="false">MIN(B5:B10)</f>
+      <c r="D10" s="43" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="49" t="s">
+        <v>194</v>
+      </c>
+      <c r="B11" s="50" t="n">
+        <f aca="false">Sparhebel!B40</f>
         <v>396.91</v>
       </c>
-      <c r="D13" s="37" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="22" t="s">
-        <v>109</v>
-      </c>
-      <c r="B14" s="36" t="n">
-        <f aca="false">B5-MIN(B5:B10)</f>
+      <c r="C11" s="51" t="n">
+        <f aca="false">$B$5-B11</f>
         <v>503.08</v>
       </c>
+      <c r="D11" s="52" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="47" t="s">
+        <v>196</v>
+      </c>
+      <c r="B12" s="48" t="n">
+        <f aca="false">Sparhebel!B41</f>
+        <v>218.6304</v>
+      </c>
+      <c r="C12" s="27" t="n">
+        <f aca="false">$B$5-B12</f>
+        <v>681.3596</v>
+      </c>
+      <c r="D12" s="43" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="3" t="s">
+        <v>198</v>
+      </c>
+      <c r="B14" s="4"/>
+      <c r="C14" s="4"/>
+      <c r="D14" s="4"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="0" t="s">
-        <v>110</v>
-      </c>
-      <c r="B15" s="14" t="n">
-        <f aca="false">(B5-MIN(B5:B10))/B5</f>
+      <c r="A15" s="24" t="s">
+        <v>199</v>
+      </c>
+      <c r="B15" s="46" t="n">
+        <f aca="false">MIN(B5:B11)</f>
+        <v>396.91</v>
+      </c>
+      <c r="D15" s="53" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="6" t="s">
+        <v>201</v>
+      </c>
+      <c r="B16" s="54" t="n">
+        <f aca="false">B5-MIN(B5:B11)</f>
+        <v>503.08</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="6" t="s">
+        <v>202</v>
+      </c>
+      <c r="B17" s="15" t="n">
+        <f aca="false">(B5-MIN(B5:B11))/B5</f>
         <v>0.558983988710986</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="18" t="s">
-        <v>111</v>
-      </c>
-      <c r="B17" s="18"/>
-      <c r="C17" s="18"/>
-      <c r="D17" s="18"/>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="24" t="s">
+        <v>203</v>
+      </c>
+      <c r="B18" s="55" t="n">
+        <f aca="false">MIN(B5:B12)</f>
+        <v>218.6304</v>
+      </c>
+      <c r="D18" s="53" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="20" t="s">
+        <v>205</v>
+      </c>
+      <c r="B20" s="20"/>
+      <c r="C20" s="20"/>
+      <c r="D20" s="20"/>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A17:D17"/>
+    <mergeCell ref="A20:D20"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>